<commit_message>
pequeña modificacion en busqueda local
</commit_message>
<xml_diff>
--- a/Tablas_MH2026.xlsx
+++ b/Tablas_MH2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pablo\Downloads\Ing.Informatica\Tercer Curso\Primer Cuatri\Meta\Practicas\Practica1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2030D8D-BDB9-4022-9745-97E5EC173B0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2699788-6F28-4F42-BEC4-7037DFACBF84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -804,7 +804,8 @@
     <col min="4" max="4" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.5546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.6640625" bestFit="1" customWidth="1"/>
@@ -1320,8 +1321,12 @@
       <c r="E19" s="17">
         <v>0.21149999999999999</v>
       </c>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
+      <c r="F19" s="17">
+        <v>51649788.170000002</v>
+      </c>
+      <c r="G19" s="17">
+        <v>109988455.09999999</v>
+      </c>
       <c r="H19" s="17">
         <v>603251.89</v>
       </c>
@@ -1357,11 +1362,11 @@
       </c>
       <c r="F20" s="18">
         <f>AVERAGE((F17-G$3)/G$3,(F18-G$3)/G$3,(F19-G$3)/G$3)</f>
-        <v>51.76828478277266</v>
+        <v>78.450836115252557</v>
       </c>
       <c r="G20" s="19">
         <f>AVERAGE(G17:G19)</f>
-        <v>110690.89199999999</v>
+        <v>36736612.294666663</v>
       </c>
       <c r="H20" s="18">
         <f>AVERAGE((H17-I$3)/I$3,(H18-I$3)/I$3,(H19-I$3)/I$3)</f>
@@ -1402,11 +1407,11 @@
       </c>
       <c r="F21" s="19">
         <f>STDEV((F17-G$3)/G$3,(F18-G$3)/G$3,(F19-G$3)/G$3)</f>
-        <v>45.69904373978946</v>
+        <v>0.54848266400633539</v>
       </c>
       <c r="G21" s="19">
         <f>STDEV(G17:G19)</f>
-        <v>1196.7567311120813</v>
+        <v>63437956.749087222</v>
       </c>
       <c r="H21" s="19">
         <f>STDEV((H17-I$3)/I$3,(H18-I$3)/I$3,(H19-I$3)/I$3)</f>
@@ -1871,11 +1876,11 @@
       </c>
       <c r="F52" s="3">
         <f>F20</f>
-        <v>51.76828478277266</v>
+        <v>78.450836115252557</v>
       </c>
       <c r="G52" s="3">
         <f>G20</f>
-        <v>110690.89199999999</v>
+        <v>36736612.294666663</v>
       </c>
       <c r="H52" s="3">
         <f>H20</f>
@@ -1895,11 +1900,11 @@
       </c>
       <c r="L52" s="8">
         <f>AVERAGE(B52,D52,F52,H52,J52)</f>
-        <v>20.691151022961638</v>
+        <v>26.027661289457619</v>
       </c>
       <c r="M52" s="8">
         <f>AVERAGE(C52,E52,G52,I52,K52)</f>
-        <v>22140.837566666662</v>
+        <v>7347325.1181000005</v>
       </c>
     </row>
     <row r="53" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>